<commit_message>
rebuilding my conference_features.json and my conference_weights.json in order to aline it with all my file. improvement of all parse_external by adding code to send file in "data/processed/external"
</commit_message>
<xml_diff>
--- a/DatasetStructure.xlsx
+++ b/DatasetStructure.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\Document Personnel\BI Microsoft\CodePython\Exorepeateone\Exo Baby names Us\Georgia Tech\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{090F85C7-CD81-4797-AB19-033D951E35D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42804292-1DB8-4BF7-B66E-2F4C46364102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="20" windowWidth="38620" windowHeight="21820" activeTab="6" xr2:uid="{FE357E66-ED91-4D96-BB26-63458C1F6D40}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="7" xr2:uid="{FE357E66-ED91-4D96-BB26-63458C1F6D40}"/>
   </bookViews>
   <sheets>
     <sheet name="Info Match" sheetId="1" r:id="rId1"/>
@@ -20,9 +20,10 @@
     <sheet name="Média &amp; Assets" sheetId="5" r:id="rId5"/>
     <sheet name="Colonnes Techniques" sheetId="6" r:id="rId6"/>
     <sheet name="Liste des scrapers" sheetId="7" r:id="rId7"/>
+    <sheet name="Conference" sheetId="8" r:id="rId8"/>
+    <sheet name="Sheet2" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="125">
   <si>
     <t xml:space="preserve">Colonne </t>
   </si>
@@ -337,6 +338,87 @@
   </si>
   <si>
     <t xml:space="preserve">Classements des prospects </t>
+  </si>
+  <si>
+    <t>Metric</t>
+  </si>
+  <si>
+    <t>CFBD API</t>
+  </si>
+  <si>
+    <t>Source officielle</t>
+  </si>
+  <si>
+    <t>Dossier</t>
+  </si>
+  <si>
+    <t>EPA</t>
+  </si>
+  <si>
+    <t>❌</t>
+  </si>
+  <si>
+    <t>CfbfastR</t>
+  </si>
+  <si>
+    <t>raw/epa.csv</t>
+  </si>
+  <si>
+    <t>Recruiting</t>
+  </si>
+  <si>
+    <t>247Sports</t>
+  </si>
+  <si>
+    <t>raw/recruiting.csv</t>
+  </si>
+  <si>
+    <t>NFL</t>
+  </si>
+  <si>
+    <t>Pro Football Reference</t>
+  </si>
+  <si>
+    <t>raw/nfl.csv</t>
+  </si>
+  <si>
+    <t>TV Ratings</t>
+  </si>
+  <si>
+    <t>SportsMediaWatch</t>
+  </si>
+  <si>
+    <t>raw/tv.csv</t>
+  </si>
+  <si>
+    <t>Top25</t>
+  </si>
+  <si>
+    <t>AP News</t>
+  </si>
+  <si>
+    <t>raw/top25.csv</t>
+  </si>
+  <si>
+    <t>Coaching</t>
+  </si>
+  <si>
+    <t>Sports‑Reference CFB</t>
+  </si>
+  <si>
+    <t>raw/coaching.csv</t>
+  </si>
+  <si>
+    <t>Interconference</t>
+  </si>
+  <si>
+    <t>⚠️ partiel</t>
+  </si>
+  <si>
+    <t>CFBD + reconstruction</t>
+  </si>
+  <si>
+    <t>raw/interconference.csv</t>
   </si>
 </sst>
 </file>
@@ -1220,4 +1302,139 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{681F6610-784C-492D-BE5C-27CDCE2C1AA1}">
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="2" max="2" width="24.6640625" customWidth="1"/>
+    <col min="3" max="3" width="23.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1" t="s">
+        <v>100</v>
+      </c>
+      <c r="D1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C4" t="s">
+        <v>110</v>
+      </c>
+      <c r="D4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" t="s">
+        <v>113</v>
+      </c>
+      <c r="D5" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C6" t="s">
+        <v>116</v>
+      </c>
+      <c r="D6" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
+        <v>118</v>
+      </c>
+      <c r="B7" t="s">
+        <v>103</v>
+      </c>
+      <c r="C7" t="s">
+        <v>119</v>
+      </c>
+      <c r="D7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B8" t="s">
+        <v>122</v>
+      </c>
+      <c r="C8" t="s">
+        <v>123</v>
+      </c>
+      <c r="D8" t="s">
+        <v>124</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE4418E4-2B09-4F51-84B6-8110DABF2DAE}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>